<commit_message>
Render line families at full size: every thin line 1 mm x 40 mm
Families 1-6 now use the measured master scale (1.0 instead of 0.9), so
their shafts are 1 mm thick and 40 mm long (80 mm extended), identical
to the plain-line control; endpoints scale with them. The SVG artwork
is unchanged. The train (0.6) and lamp (0.75) keep their size because
at full size they do not fit the fixed 220 x 120 mm stage.

Stimulus set and layout version bumped to 2026-10-07-unit-lines-v2;
data files, notation spreadsheet, specification, PDF and tests updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011vBMpHHHFiFuo75D5irsrx
</commit_message>
<xml_diff>
--- a/data/stimuli-notation.xlsx
+++ b/data/stimuli-notation.xlsx
@@ -1062,10 +1062,10 @@
         </is>
       </c>
       <c r="K5" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
@@ -1073,16 +1073,16 @@
         </is>
       </c>
       <c r="N5" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
@@ -1141,10 +1141,10 @@
         </is>
       </c>
       <c r="K6" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
@@ -1152,16 +1152,16 @@
         </is>
       </c>
       <c r="N6" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="Q6" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
@@ -1220,10 +1220,10 @@
         </is>
       </c>
       <c r="K7" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
@@ -1231,16 +1231,16 @@
         </is>
       </c>
       <c r="N7" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
@@ -1299,10 +1299,10 @@
         </is>
       </c>
       <c r="K8" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
@@ -1310,16 +1310,16 @@
         </is>
       </c>
       <c r="N8" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R8" s="5" t="inlineStr">
         <is>
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="K9" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
@@ -1389,16 +1389,16 @@
         </is>
       </c>
       <c r="N9" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
@@ -1457,10 +1457,10 @@
         </is>
       </c>
       <c r="K10" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
@@ -1468,16 +1468,16 @@
         </is>
       </c>
       <c r="N10" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R10" s="5" t="inlineStr">
         <is>
@@ -1536,10 +1536,10 @@
         </is>
       </c>
       <c r="K11" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
@@ -1547,16 +1547,16 @@
         </is>
       </c>
       <c r="N11" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
@@ -1615,10 +1615,10 @@
         </is>
       </c>
       <c r="K12" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
@@ -1626,16 +1626,16 @@
         </is>
       </c>
       <c r="N12" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R12" s="5" t="inlineStr">
         <is>
@@ -1694,10 +1694,10 @@
         </is>
       </c>
       <c r="K13" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
@@ -1705,16 +1705,16 @@
         </is>
       </c>
       <c r="N13" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>39.6</v>
+        <v>44</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="R13" s="5" t="inlineStr">
         <is>
@@ -1773,10 +1773,10 @@
         </is>
       </c>
       <c r="K14" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
@@ -1784,16 +1784,16 @@
         </is>
       </c>
       <c r="N14" s="5" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>43.2</v>
+        <v>48</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
@@ -1856,10 +1856,10 @@
         </is>
       </c>
       <c r="K15" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
@@ -1867,16 +1867,16 @@
         </is>
       </c>
       <c r="N15" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>75.59999999999999</v>
+        <v>84</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
@@ -1935,10 +1935,10 @@
         </is>
       </c>
       <c r="K16" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
@@ -1946,16 +1946,16 @@
         </is>
       </c>
       <c r="N16" s="5" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>79.2</v>
+        <v>88</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="R16" s="5" t="inlineStr">
         <is>
@@ -2014,10 +2014,10 @@
         </is>
       </c>
       <c r="K17" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M17" s="5" t="inlineStr">
         <is>
@@ -2025,16 +2025,16 @@
         </is>
       </c>
       <c r="N17" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>37.8</v>
+        <v>42</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="R17" s="5" t="inlineStr">
         <is>
@@ -2093,10 +2093,10 @@
         </is>
       </c>
       <c r="K18" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
@@ -2104,16 +2104,16 @@
         </is>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>37.8</v>
+        <v>42</v>
       </c>
       <c r="Q18" s="5" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="R18" s="5" t="inlineStr">
         <is>
@@ -2176,10 +2176,10 @@
         </is>
       </c>
       <c r="K19" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
@@ -2187,16 +2187,16 @@
         </is>
       </c>
       <c r="N19" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>73.8</v>
+        <v>82</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="R19" s="5" t="inlineStr">
         <is>
@@ -2255,10 +2255,10 @@
         </is>
       </c>
       <c r="K20" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
@@ -2266,16 +2266,16 @@
         </is>
       </c>
       <c r="N20" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="P20" s="5" t="n">
-        <v>75.59999999999999</v>
+        <v>84</v>
       </c>
       <c r="Q20" s="5" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="R20" s="5" t="inlineStr">
         <is>
@@ -2334,10 +2334,10 @@
         </is>
       </c>
       <c r="K21" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
@@ -2345,16 +2345,16 @@
         </is>
       </c>
       <c r="N21" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O21" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P21" s="5" t="n">
-        <v>40.5</v>
+        <v>45</v>
       </c>
       <c r="Q21" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="R21" s="5" t="inlineStr">
         <is>
@@ -2417,10 +2417,10 @@
         </is>
       </c>
       <c r="K22" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
         </is>
       </c>
       <c r="N22" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O22" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P22" s="5" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="Q22" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R22" s="5" t="inlineStr">
         <is>
@@ -2496,10 +2496,10 @@
         </is>
       </c>
       <c r="K23" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
@@ -2507,16 +2507,16 @@
         </is>
       </c>
       <c r="N23" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="O23" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="P23" s="5" t="n">
-        <v>76.5</v>
+        <v>85</v>
       </c>
       <c r="Q23" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="R23" s="5" t="inlineStr">
         <is>
@@ -2575,10 +2575,10 @@
         </is>
       </c>
       <c r="K24" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
@@ -2586,16 +2586,16 @@
         </is>
       </c>
       <c r="N24" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O24" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P24" s="5" t="n">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="Q24" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R24" s="5" t="inlineStr">
         <is>
@@ -2654,10 +2654,10 @@
         </is>
       </c>
       <c r="K25" s="5" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
@@ -2665,16 +2665,16 @@
         </is>
       </c>
       <c r="N25" s="5" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="O25" s="5" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="P25" s="5" t="n">
-        <v>43.2</v>
+        <v>48</v>
       </c>
       <c r="Q25" s="5" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="R25" s="5" t="inlineStr">
         <is>
@@ -2733,10 +2733,10 @@
         </is>
       </c>
       <c r="K26" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
@@ -2744,16 +2744,16 @@
         </is>
       </c>
       <c r="N26" s="5" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
       <c r="O26" s="5" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="P26" s="5" t="n">
-        <v>79.2</v>
+        <v>88</v>
       </c>
       <c r="Q26" s="5" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="R26" s="5" t="inlineStr">
         <is>
@@ -2816,10 +2816,10 @@
         </is>
       </c>
       <c r="K27" s="5" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L27" s="5" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
@@ -2827,16 +2827,16 @@
         </is>
       </c>
       <c r="N27" s="5" t="n">
-        <v>14.4</v>
+        <v>16</v>
       </c>
       <c r="O27" s="5" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="P27" s="5" t="n">
-        <v>86.40000000000001</v>
+        <v>96</v>
       </c>
       <c r="Q27" s="5" t="n">
-        <v>10.8</v>
+        <v>12</v>
       </c>
       <c r="R27" s="5" t="inlineStr">
         <is>

</xml_diff>